<commit_message>
Fix image recognition bugs
</commit_message>
<xml_diff>
--- a/Dune_Imperium_Card_Inventory.xlsx
+++ b/Dune_Imperium_Card_Inventory.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Imperium" sheetId="1" state="visible" r:id="rId2"/>
@@ -2470,7 +2470,7 @@
     <t xml:space="preserve">If you have a seat on the High Council and 2 DNA: +1 Victory Point</t>
   </si>
   <si>
-    <t xml:space="preserve">To the Victor …</t>
+    <t xml:space="preserve">To the Victor…</t>
   </si>
   <si>
     <t xml:space="preserve">When you win a Conflict: +3 Spice.
@@ -5809,7 +5809,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AK186"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="15"/>
@@ -18020,7 +18020,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O19"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
@@ -18714,7 +18714,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:AB999"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="16.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="16.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.71"/>
@@ -49239,7 +49239,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P1000"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.3"/>
@@ -53396,7 +53396,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AG20"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
@@ -54720,7 +54720,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:V6"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
@@ -55148,7 +55148,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R132"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="4" style="0" width="14.29"/>
@@ -59500,7 +59500,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M37"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.86"/>
@@ -60601,7 +60601,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E37"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.29"/>
@@ -61240,7 +61240,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D37"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="15"/>
@@ -61573,7 +61573,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Y11"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="97.57"/>
   </cols>
@@ -61675,7 +61675,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H33"/>
-  <sheetFormatPr defaultColWidth="14.49609375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="14.5" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="26.57"/>

</xml_diff>